<commit_message>
Linear combination up to three organisms
</commit_message>
<xml_diff>
--- a/Spectral_library.xlsx
+++ b/Spectral_library.xlsx
@@ -1,36 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vunl-my.sharepoint.com/personal/v_u_chukhutsina_vu_nl/Documents/TenureTrack/ML_project_photosynthesis/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a4d4da14dbd511bc/Documents/Mats/UvA/Master/Machine Learning/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{BF98154F-B8E6-7849-B853-90E5BF6286B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4AC0A54-D01C-944A-B23E-997EDBB67239}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{BF98154F-B8E6-7849-B853-90E5BF6286B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78F0CB8D-56D5-42E8-AC87-833B23DF4C15}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="640" windowWidth="34560" windowHeight="20860" xr2:uid="{B2930DF6-989B-44EA-8F1B-19D5C9138BC6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B2930DF6-989B-44EA-8F1B-19D5C9138BC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -66,13 +55,13 @@
     <t>Dinoflagellate_Smicroadriaticum</t>
   </si>
   <si>
-    <t>Dinoflagelalte_Dtrenchii</t>
-  </si>
-  <si>
     <t>Dinoflagellate_Cgoreaui</t>
   </si>
   <si>
     <t>Cyanobacteria_Synechosystis</t>
+  </si>
+  <si>
+    <t>Dinoflagellate_Dtrenchii</t>
   </si>
 </sst>
 </file>
@@ -446,12 +435,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{985166C8-05CF-4B35-AFB5-F783E4CB5F67}">
   <dimension ref="A1:Q463"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="8.5" customWidth="1"/>
+    <col min="2" max="2" width="8.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -483,19 +472,19 @@
         <v>8</v>
       </c>
       <c r="M1" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" t="s">
         <v>9</v>
-      </c>
-      <c r="N1" t="s">
-        <v>10</v>
       </c>
       <c r="P1" t="s">
         <v>0</v>
       </c>
       <c r="Q1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>700</v>
       </c>
@@ -539,7 +528,7 @@
         <v>-6.7402399999999996E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>699</v>
       </c>
@@ -583,7 +572,7 @@
         <v>-4.6487200000000002E-4</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>698</v>
       </c>
@@ -627,7 +616,7 @@
         <v>2.1418199999999999E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>697</v>
       </c>
@@ -671,7 +660,7 @@
         <v>3.13818E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>696</v>
       </c>
@@ -715,7 +704,7 @@
         <v>1.3396099999999999E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>695</v>
       </c>
@@ -759,7 +748,7 @@
         <v>8.8132899999999998E-5</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>694</v>
       </c>
@@ -803,7 +792,7 @@
         <v>-8.1285799999999993E-5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>693</v>
       </c>
@@ -847,7 +836,7 @@
         <v>-1.53907E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>692</v>
       </c>
@@ -891,7 +880,7 @@
         <v>-1.9614400000000001E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>691</v>
       </c>
@@ -935,7 +924,7 @@
         <v>-1.53609E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>690</v>
       </c>
@@ -979,7 +968,7 @@
         <v>2.24754E-4</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>689</v>
       </c>
@@ -1023,7 +1012,7 @@
         <v>4.7569000000000002E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>688</v>
       </c>
@@ -1067,7 +1056,7 @@
         <v>1.3600999999999999E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>687</v>
       </c>
@@ -1111,7 +1100,7 @@
         <v>4.0265899999999998E-4</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>686</v>
       </c>
@@ -1155,7 +1144,7 @@
         <v>-1.9461700000000001E-4</v>
       </c>
     </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>685</v>
       </c>
@@ -1199,7 +1188,7 @@
         <v>2.9198799999999999E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>684</v>
       </c>
@@ -1243,7 +1232,7 @@
         <v>5.6773400000000001E-5</v>
       </c>
     </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>683</v>
       </c>
@@ -1287,7 +1276,7 @@
         <v>-7.8839800000000005E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>682</v>
       </c>
@@ -1331,7 +1320,7 @@
         <v>-5.9664199999999997E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>681</v>
       </c>
@@ -1375,7 +1364,7 @@
         <v>4.06504E-5</v>
       </c>
     </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>680</v>
       </c>
@@ -1419,7 +1408,7 @@
         <v>2.8105799999999999E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>679</v>
       </c>
@@ -1463,7 +1452,7 @@
         <v>4.3930100000000001E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>678</v>
       </c>
@@ -1507,7 +1496,7 @@
         <v>-5.0157300000000002E-5</v>
       </c>
     </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>677</v>
       </c>
@@ -1551,7 +1540,7 @@
         <v>-4.1072800000000002E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>676</v>
       </c>
@@ -1595,7 +1584,7 @@
         <v>-3.2858600000000001E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>675</v>
       </c>
@@ -1639,7 +1628,7 @@
         <v>-4.62502E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>674</v>
       </c>
@@ -1683,7 +1672,7 @@
         <v>-6.4708299999999998E-5</v>
       </c>
     </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>673</v>
       </c>
@@ -1727,7 +1716,7 @@
         <v>-1.33194E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>672</v>
       </c>
@@ -1771,7 +1760,7 @@
         <v>-4.2107000000000001E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>671</v>
       </c>
@@ -1815,7 +1804,7 @@
         <v>-4.0479000000000003E-5</v>
       </c>
     </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>670</v>
       </c>
@@ -1859,7 +1848,7 @@
         <v>-2.2132E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>669</v>
       </c>
@@ -1903,7 +1892,7 @@
         <v>-5.9621000000000001E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>668</v>
       </c>
@@ -1947,7 +1936,7 @@
         <v>-5.6795800000000003E-5</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>667</v>
       </c>
@@ -1991,7 +1980,7 @@
         <v>2.6021200000000001E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>666</v>
       </c>
@@ -2035,7 +2024,7 @@
         <v>4.1909500000000003E-5</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>665</v>
       </c>
@@ -2079,7 +2068,7 @@
         <v>3.0851400000000002E-4</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>664</v>
       </c>
@@ -2123,7 +2112,7 @@
         <v>3.0142100000000001E-4</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>663</v>
       </c>
@@ -2167,7 +2156,7 @@
         <v>-3.81596E-4</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>662</v>
       </c>
@@ -2211,7 +2200,7 @@
         <v>-1.4764800000000001E-4</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>661</v>
       </c>
@@ -2255,7 +2244,7 @@
         <v>-7.1065099999999997E-4</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>660</v>
       </c>
@@ -2299,7 +2288,7 @@
         <v>-5.31077E-5</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>659</v>
       </c>
@@ -2343,7 +2332,7 @@
         <v>-4.1827599999999998E-4</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>658</v>
       </c>
@@ -2387,7 +2376,7 @@
         <v>2.7041100000000002E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>657</v>
       </c>
@@ -2431,7 +2420,7 @@
         <v>-3.4499900000000002E-4</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>656</v>
       </c>
@@ -2475,7 +2464,7 @@
         <v>3.7572499999999998E-4</v>
       </c>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>655</v>
       </c>
@@ -2519,7 +2508,7 @@
         <v>3.81052E-4</v>
       </c>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>654</v>
       </c>
@@ -2563,7 +2552,7 @@
         <v>-8.7462399999999998E-5</v>
       </c>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>653</v>
       </c>
@@ -2607,7 +2596,7 @@
         <v>1.1228E-4</v>
       </c>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>652</v>
       </c>
@@ -2651,7 +2640,7 @@
         <v>1.17518E-4</v>
       </c>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>651</v>
       </c>
@@ -2695,7 +2684,7 @@
         <v>5.2365699999999996E-4</v>
       </c>
     </row>
-    <row r="52" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>650</v>
       </c>
@@ -2739,7 +2728,7 @@
         <v>2.6554600000000002E-4</v>
       </c>
     </row>
-    <row r="53" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>649</v>
       </c>
@@ -2783,7 +2772,7 @@
         <v>4.28751E-4</v>
       </c>
     </row>
-    <row r="54" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>648</v>
       </c>
@@ -2827,7 +2816,7 @@
         <v>-9.5881499999999993E-5</v>
       </c>
     </row>
-    <row r="55" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>647</v>
       </c>
@@ -2871,7 +2860,7 @@
         <v>-1.2698000000000001E-4</v>
       </c>
     </row>
-    <row r="56" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>646</v>
       </c>
@@ -2915,7 +2904,7 @@
         <v>3.06457E-4</v>
       </c>
     </row>
-    <row r="57" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>645</v>
       </c>
@@ -2959,7 +2948,7 @@
         <v>4.7184500000000002E-5</v>
       </c>
     </row>
-    <row r="58" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>644</v>
       </c>
@@ -3003,7 +2992,7 @@
         <v>2.4875299999999999E-4</v>
       </c>
     </row>
-    <row r="59" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>643</v>
       </c>
@@ -3047,7 +3036,7 @@
         <v>5.0874799999999995E-4</v>
       </c>
     </row>
-    <row r="60" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>642</v>
       </c>
@@ -3091,7 +3080,7 @@
         <v>3.3105899999999998E-4</v>
       </c>
     </row>
-    <row r="61" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>641</v>
       </c>
@@ -3135,7 +3124,7 @@
         <v>5.5380200000000005E-4</v>
       </c>
     </row>
-    <row r="62" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>640</v>
       </c>
@@ -3179,7 +3168,7 @@
         <v>1.09E-3</v>
       </c>
     </row>
-    <row r="63" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>639</v>
       </c>
@@ -3223,7 +3212,7 @@
         <v>8.4403899999999999E-4</v>
       </c>
     </row>
-    <row r="64" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>638</v>
       </c>
@@ -3267,7 +3256,7 @@
         <v>3.8589499999999998E-4</v>
       </c>
     </row>
-    <row r="65" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>637</v>
       </c>
@@ -3311,7 +3300,7 @@
         <v>4.6965499999999997E-4</v>
       </c>
     </row>
-    <row r="66" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>636</v>
       </c>
@@ -3355,7 +3344,7 @@
         <v>4.0343399999999999E-4</v>
       </c>
     </row>
-    <row r="67" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>635</v>
       </c>
@@ -3399,7 +3388,7 @@
         <v>6.6892799999999995E-4</v>
       </c>
     </row>
-    <row r="68" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>634</v>
       </c>
@@ -3443,7 +3432,7 @@
         <v>6.8116900000000002E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>633</v>
       </c>
@@ -3487,7 +3476,7 @@
         <v>6.2764400000000001E-4</v>
       </c>
     </row>
-    <row r="70" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>632</v>
       </c>
@@ -3531,7 +3520,7 @@
         <v>8.16889E-4</v>
       </c>
     </row>
-    <row r="71" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>631</v>
       </c>
@@ -3575,7 +3564,7 @@
         <v>1.39E-3</v>
       </c>
     </row>
-    <row r="72" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>630</v>
       </c>
@@ -3619,7 +3608,7 @@
         <v>1.39E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>629</v>
       </c>
@@ -3663,7 +3652,7 @@
         <v>1.48E-3</v>
       </c>
     </row>
-    <row r="74" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>628</v>
       </c>
@@ -3707,7 +3696,7 @@
         <v>1.6299999999999999E-3</v>
       </c>
     </row>
-    <row r="75" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>627</v>
       </c>
@@ -3751,7 +3740,7 @@
         <v>1.4599999999999999E-3</v>
       </c>
     </row>
-    <row r="76" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>626</v>
       </c>
@@ -3795,7 +3784,7 @@
         <v>1.9499999999999999E-3</v>
       </c>
     </row>
-    <row r="77" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>625</v>
       </c>
@@ -3839,7 +3828,7 @@
         <v>2.16E-3</v>
       </c>
     </row>
-    <row r="78" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>624</v>
       </c>
@@ -3883,7 +3872,7 @@
         <v>2.3E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>623</v>
       </c>
@@ -3927,7 +3916,7 @@
         <v>2.6700000000000001E-3</v>
       </c>
     </row>
-    <row r="80" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>622</v>
       </c>
@@ -3971,7 +3960,7 @@
         <v>3.46E-3</v>
       </c>
     </row>
-    <row r="81" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>621</v>
       </c>
@@ -4015,7 +4004,7 @@
         <v>3.8700000000000002E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>620</v>
       </c>
@@ -4059,7 +4048,7 @@
         <v>4.2199999999999998E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>619</v>
       </c>
@@ -4103,7 +4092,7 @@
         <v>5.1599999999999997E-3</v>
       </c>
     </row>
-    <row r="84" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>618</v>
       </c>
@@ -4147,7 +4136,7 @@
         <v>5.77E-3</v>
       </c>
     </row>
-    <row r="85" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>617</v>
       </c>
@@ -4191,7 +4180,7 @@
         <v>6.5399999999999998E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>616</v>
       </c>
@@ -4235,7 +4224,7 @@
         <v>6.7999999999999996E-3</v>
       </c>
     </row>
-    <row r="87" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>615</v>
       </c>
@@ -4279,7 +4268,7 @@
         <v>8.1700000000000002E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>614</v>
       </c>
@@ -4323,7 +4312,7 @@
         <v>8.9800000000000001E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>613</v>
       </c>
@@ -4367,7 +4356,7 @@
         <v>9.9500000000000005E-3</v>
       </c>
     </row>
-    <row r="90" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>612</v>
       </c>
@@ -4411,7 +4400,7 @@
         <v>1.1350000000000001E-2</v>
       </c>
     </row>
-    <row r="91" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>611</v>
       </c>
@@ -4455,7 +4444,7 @@
         <v>1.274E-2</v>
       </c>
     </row>
-    <row r="92" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>610</v>
       </c>
@@ -4499,7 +4488,7 @@
         <v>1.418E-2</v>
       </c>
     </row>
-    <row r="93" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>609</v>
       </c>
@@ -4543,7 +4532,7 @@
         <v>1.5769999999999999E-2</v>
       </c>
     </row>
-    <row r="94" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>608</v>
       </c>
@@ -4587,7 +4576,7 @@
         <v>1.7729999999999999E-2</v>
       </c>
     </row>
-    <row r="95" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>607</v>
       </c>
@@ -4631,7 +4620,7 @@
         <v>1.9820000000000001E-2</v>
       </c>
     </row>
-    <row r="96" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>606</v>
       </c>
@@ -4675,7 +4664,7 @@
         <v>2.1690000000000001E-2</v>
       </c>
     </row>
-    <row r="97" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>605</v>
       </c>
@@ -4719,7 +4708,7 @@
         <v>2.3769999999999999E-2</v>
       </c>
     </row>
-    <row r="98" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>604</v>
       </c>
@@ -4763,7 +4752,7 @@
         <v>2.6530000000000001E-2</v>
       </c>
     </row>
-    <row r="99" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>603</v>
       </c>
@@ -4807,7 +4796,7 @@
         <v>2.8819999999999998E-2</v>
       </c>
     </row>
-    <row r="100" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>602</v>
       </c>
@@ -4851,7 +4840,7 @@
         <v>3.1629999999999998E-2</v>
       </c>
     </row>
-    <row r="101" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>601</v>
       </c>
@@ -4895,7 +4884,7 @@
         <v>3.4590000000000003E-2</v>
       </c>
     </row>
-    <row r="102" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>600</v>
       </c>
@@ -4939,7 +4928,7 @@
         <v>3.8109999999999998E-2</v>
       </c>
     </row>
-    <row r="103" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>599</v>
       </c>
@@ -4983,7 +4972,7 @@
         <v>4.2070000000000003E-2</v>
       </c>
     </row>
-    <row r="104" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>598</v>
       </c>
@@ -5027,7 +5016,7 @@
         <v>4.6929999999999999E-2</v>
       </c>
     </row>
-    <row r="105" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>597</v>
       </c>
@@ -5071,7 +5060,7 @@
         <v>5.1580000000000001E-2</v>
       </c>
     </row>
-    <row r="106" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>596</v>
       </c>
@@ -5115,7 +5104,7 @@
         <v>5.7259999999999998E-2</v>
       </c>
     </row>
-    <row r="107" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>595</v>
       </c>
@@ -5159,7 +5148,7 @@
         <v>6.4009999999999997E-2</v>
       </c>
     </row>
-    <row r="108" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>594</v>
       </c>
@@ -5203,7 +5192,7 @@
         <v>7.1429999999999993E-2</v>
       </c>
     </row>
-    <row r="109" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>593</v>
       </c>
@@ -5247,7 +5236,7 @@
         <v>7.9409999999999994E-2</v>
       </c>
     </row>
-    <row r="110" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>592</v>
       </c>
@@ -5291,7 +5280,7 @@
         <v>8.9289999999999994E-2</v>
       </c>
     </row>
-    <row r="111" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>591</v>
       </c>
@@ -5335,7 +5324,7 @@
         <v>9.937E-2</v>
       </c>
     </row>
-    <row r="112" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>590</v>
       </c>
@@ -5379,7 +5368,7 @@
         <v>0.11022</v>
       </c>
     </row>
-    <row r="113" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>589</v>
       </c>
@@ -5423,7 +5412,7 @@
         <v>0.12186</v>
       </c>
     </row>
-    <row r="114" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>588</v>
       </c>
@@ -5467,7 +5456,7 @@
         <v>0.13303000000000001</v>
       </c>
     </row>
-    <row r="115" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>587</v>
       </c>
@@ -5511,7 +5500,7 @@
         <v>0.14435000000000001</v>
       </c>
     </row>
-    <row r="116" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>586</v>
       </c>
@@ -5555,7 +5544,7 @@
         <v>0.15498999999999999</v>
       </c>
     </row>
-    <row r="117" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>585</v>
       </c>
@@ -5599,7 +5588,7 @@
         <v>0.16458999999999999</v>
       </c>
     </row>
-    <row r="118" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>584</v>
       </c>
@@ -5643,7 +5632,7 @@
         <v>0.17276</v>
       </c>
     </row>
-    <row r="119" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>583</v>
       </c>
@@ -5687,7 +5676,7 @@
         <v>0.17951</v>
       </c>
     </row>
-    <row r="120" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>582</v>
       </c>
@@ -5731,7 +5720,7 @@
         <v>0.18468000000000001</v>
       </c>
     </row>
-    <row r="121" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>581</v>
       </c>
@@ -5775,7 +5764,7 @@
         <v>0.18833</v>
       </c>
     </row>
-    <row r="122" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>580</v>
       </c>
@@ -5819,7 +5808,7 @@
         <v>0.18992000000000001</v>
       </c>
     </row>
-    <row r="123" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>579</v>
       </c>
@@ -5863,7 +5852,7 @@
         <v>0.19023000000000001</v>
       </c>
     </row>
-    <row r="124" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>578</v>
       </c>
@@ -5907,7 +5896,7 @@
         <v>0.18917</v>
       </c>
     </row>
-    <row r="125" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>577</v>
       </c>
@@ -5951,7 +5940,7 @@
         <v>0.18779999999999999</v>
       </c>
     </row>
-    <row r="126" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>576</v>
       </c>
@@ -5995,7 +5984,7 @@
         <v>0.18543999999999999</v>
       </c>
     </row>
-    <row r="127" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>575</v>
       </c>
@@ -6039,7 +6028,7 @@
         <v>0.18343999999999999</v>
       </c>
     </row>
-    <row r="128" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>574</v>
       </c>
@@ -6083,7 +6072,7 @@
         <v>0.18079999999999999</v>
       </c>
     </row>
-    <row r="129" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>573</v>
       </c>
@@ -6127,7 +6116,7 @@
         <v>0.17817</v>
       </c>
     </row>
-    <row r="130" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>572</v>
       </c>
@@ -6171,7 +6160,7 @@
         <v>0.17559</v>
       </c>
     </row>
-    <row r="131" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>571</v>
       </c>
@@ -6215,7 +6204,7 @@
         <v>0.17227999999999999</v>
       </c>
     </row>
-    <row r="132" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>570</v>
       </c>
@@ -6259,7 +6248,7 @@
         <v>0.16891</v>
       </c>
     </row>
-    <row r="133" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>569</v>
       </c>
@@ -6303,7 +6292,7 @@
         <v>0.16466</v>
       </c>
     </row>
-    <row r="134" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>568</v>
       </c>
@@ -6347,7 +6336,7 @@
         <v>0.16070000000000001</v>
       </c>
     </row>
-    <row r="135" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>567</v>
       </c>
@@ -6391,7 +6380,7 @@
         <v>0.15626000000000001</v>
       </c>
     </row>
-    <row r="136" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>566</v>
       </c>
@@ -6435,7 +6424,7 @@
         <v>0.15135000000000001</v>
       </c>
     </row>
-    <row r="137" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>565</v>
       </c>
@@ -6479,7 +6468,7 @@
         <v>0.14749999999999999</v>
       </c>
     </row>
-    <row r="138" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>564</v>
       </c>
@@ -6523,7 +6512,7 @@
         <v>0.1431</v>
       </c>
     </row>
-    <row r="139" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>563</v>
       </c>
@@ -6567,7 +6556,7 @@
         <v>0.13941000000000001</v>
       </c>
     </row>
-    <row r="140" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>562</v>
       </c>
@@ -6611,7 +6600,7 @@
         <v>0.13616</v>
       </c>
     </row>
-    <row r="141" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>561</v>
       </c>
@@ -6655,7 +6644,7 @@
         <v>0.13327</v>
       </c>
     </row>
-    <row r="142" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>560</v>
       </c>
@@ -6699,7 +6688,7 @@
         <v>0.13073000000000001</v>
       </c>
     </row>
-    <row r="143" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>559</v>
       </c>
@@ -6743,7 +6732,7 @@
         <v>0.12876000000000001</v>
       </c>
     </row>
-    <row r="144" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>558</v>
       </c>
@@ -6787,7 +6776,7 @@
         <v>0.12751999999999999</v>
       </c>
     </row>
-    <row r="145" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>557</v>
       </c>
@@ -6831,7 +6820,7 @@
         <v>0.12679000000000001</v>
       </c>
     </row>
-    <row r="146" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>556</v>
       </c>
@@ -6875,7 +6864,7 @@
         <v>0.12611</v>
       </c>
     </row>
-    <row r="147" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>555</v>
       </c>
@@ -6919,7 +6908,7 @@
         <v>0.12595000000000001</v>
       </c>
     </row>
-    <row r="148" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>554</v>
       </c>
@@ -6963,7 +6952,7 @@
         <v>0.12606999999999999</v>
       </c>
     </row>
-    <row r="149" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>553</v>
       </c>
@@ -7007,7 +6996,7 @@
         <v>0.12633</v>
       </c>
     </row>
-    <row r="150" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>552</v>
       </c>
@@ -7051,7 +7040,7 @@
         <v>0.12664</v>
       </c>
     </row>
-    <row r="151" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>551</v>
       </c>
@@ -7095,7 +7084,7 @@
         <v>0.12759999999999999</v>
       </c>
     </row>
-    <row r="152" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>550</v>
       </c>
@@ -7139,7 +7128,7 @@
         <v>0.12839999999999999</v>
       </c>
     </row>
-    <row r="153" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>549</v>
       </c>
@@ -7183,7 +7172,7 @@
         <v>0.12959999999999999</v>
       </c>
     </row>
-    <row r="154" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>548</v>
       </c>
@@ -7227,7 +7216,7 @@
         <v>0.13095999999999999</v>
       </c>
     </row>
-    <row r="155" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>547</v>
       </c>
@@ -7271,7 +7260,7 @@
         <v>0.13266</v>
       </c>
     </row>
-    <row r="156" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>546</v>
       </c>
@@ -7315,7 +7304,7 @@
         <v>0.13452</v>
       </c>
     </row>
-    <row r="157" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>545</v>
       </c>
@@ -7359,7 +7348,7 @@
         <v>0.13674</v>
       </c>
     </row>
-    <row r="158" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>544</v>
       </c>
@@ -7403,7 +7392,7 @@
         <v>0.13900999999999999</v>
       </c>
     </row>
-    <row r="159" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>543</v>
       </c>
@@ -7447,7 +7436,7 @@
         <v>0.14149999999999999</v>
       </c>
     </row>
-    <row r="160" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>542</v>
       </c>
@@ -7491,7 +7480,7 @@
         <v>0.14405000000000001</v>
       </c>
     </row>
-    <row r="161" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>541</v>
       </c>
@@ -7535,7 +7524,7 @@
         <v>0.14698</v>
       </c>
     </row>
-    <row r="162" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>540</v>
       </c>
@@ -7579,7 +7568,7 @@
         <v>0.14995</v>
       </c>
     </row>
-    <row r="163" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>539</v>
       </c>
@@ -7623,7 +7612,7 @@
         <v>0.15298999999999999</v>
       </c>
     </row>
-    <row r="164" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>538</v>
       </c>
@@ -7667,7 +7656,7 @@
         <v>0.15565000000000001</v>
       </c>
     </row>
-    <row r="165" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>537</v>
       </c>
@@ -7711,7 +7700,7 @@
         <v>0.15862000000000001</v>
       </c>
     </row>
-    <row r="166" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>536</v>
       </c>
@@ -7755,7 +7744,7 @@
         <v>0.16125999999999999</v>
       </c>
     </row>
-    <row r="167" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>535</v>
       </c>
@@ -7799,7 +7788,7 @@
         <v>0.1638</v>
       </c>
     </row>
-    <row r="168" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>534</v>
       </c>
@@ -7843,7 +7832,7 @@
         <v>0.16632</v>
       </c>
     </row>
-    <row r="169" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>533</v>
       </c>
@@ -7887,7 +7876,7 @@
         <v>0.16846</v>
       </c>
     </row>
-    <row r="170" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>532</v>
       </c>
@@ -7931,7 +7920,7 @@
         <v>0.17016000000000001</v>
       </c>
     </row>
-    <row r="171" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>531</v>
       </c>
@@ -7975,7 +7964,7 @@
         <v>0.17197000000000001</v>
       </c>
     </row>
-    <row r="172" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>530</v>
       </c>
@@ -8019,7 +8008,7 @@
         <v>0.17344000000000001</v>
       </c>
     </row>
-    <row r="173" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>529</v>
       </c>
@@ -8063,7 +8052,7 @@
         <v>0.17482</v>
       </c>
     </row>
-    <row r="174" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>528</v>
       </c>
@@ -8107,7 +8096,7 @@
         <v>0.17568</v>
       </c>
     </row>
-    <row r="175" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>527</v>
       </c>
@@ -8151,7 +8140,7 @@
         <v>0.17660999999999999</v>
       </c>
     </row>
-    <row r="176" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>526</v>
       </c>
@@ -8195,7 +8184,7 @@
         <v>0.17732999999999999</v>
       </c>
     </row>
-    <row r="177" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>525</v>
       </c>
@@ -8239,7 +8228,7 @@
         <v>0.17757999999999999</v>
       </c>
     </row>
-    <row r="178" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>524</v>
       </c>
@@ -8283,7 +8272,7 @@
         <v>0.17749000000000001</v>
       </c>
     </row>
-    <row r="179" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>523</v>
       </c>
@@ -8327,7 +8316,7 @@
         <v>0.17743</v>
       </c>
     </row>
-    <row r="180" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>522</v>
       </c>
@@ -8371,7 +8360,7 @@
         <v>0.17680000000000001</v>
       </c>
     </row>
-    <row r="181" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>521</v>
       </c>
@@ -8415,7 +8404,7 @@
         <v>0.17599999999999999</v>
       </c>
     </row>
-    <row r="182" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>520</v>
       </c>
@@ -8459,7 +8448,7 @@
         <v>0.17510999999999999</v>
       </c>
     </row>
-    <row r="183" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>519</v>
       </c>
@@ -8503,7 +8492,7 @@
         <v>0.17365</v>
       </c>
     </row>
-    <row r="184" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>518</v>
       </c>
@@ -8547,7 +8536,7 @@
         <v>0.17180999999999999</v>
       </c>
     </row>
-    <row r="185" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>517</v>
       </c>
@@ -8591,7 +8580,7 @@
         <v>0.16989000000000001</v>
       </c>
     </row>
-    <row r="186" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>516</v>
       </c>
@@ -8635,7 +8624,7 @@
         <v>0.16780999999999999</v>
       </c>
     </row>
-    <row r="187" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>515</v>
       </c>
@@ -8679,7 +8668,7 @@
         <v>0.1656</v>
       </c>
     </row>
-    <row r="188" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>514</v>
       </c>
@@ -8723,7 +8712,7 @@
         <v>0.16314999999999999</v>
       </c>
     </row>
-    <row r="189" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>513</v>
       </c>
@@ -8767,7 +8756,7 @@
         <v>0.16027</v>
       </c>
     </row>
-    <row r="190" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>512</v>
       </c>
@@ -8811,7 +8800,7 @@
         <v>0.15739</v>
       </c>
     </row>
-    <row r="191" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>511</v>
       </c>
@@ -8855,7 +8844,7 @@
         <v>0.15478</v>
       </c>
     </row>
-    <row r="192" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>510</v>
       </c>
@@ -8899,7 +8888,7 @@
         <v>0.15196999999999999</v>
       </c>
     </row>
-    <row r="193" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>509</v>
       </c>
@@ -8943,7 +8932,7 @@
         <v>0.14892</v>
       </c>
     </row>
-    <row r="194" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>508</v>
       </c>
@@ -8987,7 +8976,7 @@
         <v>0.14646999999999999</v>
       </c>
     </row>
-    <row r="195" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>507</v>
       </c>
@@ -9031,7 +9020,7 @@
         <v>0.14368</v>
       </c>
     </row>
-    <row r="196" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>506</v>
       </c>
@@ -9075,7 +9064,7 @@
         <v>0.14105999999999999</v>
       </c>
     </row>
-    <row r="197" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>505</v>
       </c>
@@ -9119,7 +9108,7 @@
         <v>0.13855000000000001</v>
       </c>
     </row>
-    <row r="198" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>504</v>
       </c>
@@ -9163,7 +9152,7 @@
         <v>0.13622000000000001</v>
       </c>
     </row>
-    <row r="199" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>503</v>
       </c>
@@ -9207,7 +9196,7 @@
         <v>0.13395000000000001</v>
       </c>
     </row>
-    <row r="200" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>502</v>
       </c>
@@ -9251,7 +9240,7 @@
         <v>0.13166</v>
       </c>
     </row>
-    <row r="201" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>501</v>
       </c>
@@ -9295,7 +9284,7 @@
         <v>0.12956999999999999</v>
       </c>
     </row>
-    <row r="202" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>500</v>
       </c>
@@ -9339,7 +9328,7 @@
         <v>0.1275</v>
       </c>
     </row>
-    <row r="203" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>499</v>
       </c>
@@ -9383,7 +9372,7 @@
         <v>0.12551999999999999</v>
       </c>
     </row>
-    <row r="204" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>498</v>
       </c>
@@ -9427,7 +9416,7 @@
         <v>0.12382</v>
       </c>
     </row>
-    <row r="205" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>497</v>
       </c>
@@ -9471,7 +9460,7 @@
         <v>0.12209</v>
       </c>
     </row>
-    <row r="206" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>496</v>
       </c>
@@ -9515,7 +9504,7 @@
         <v>0.12013</v>
       </c>
     </row>
-    <row r="207" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>495</v>
       </c>
@@ -9559,7 +9548,7 @@
         <v>0.11846</v>
       </c>
     </row>
-    <row r="208" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>494</v>
       </c>
@@ -9603,7 +9592,7 @@
         <v>0.11704000000000001</v>
       </c>
     </row>
-    <row r="209" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>493</v>
       </c>
@@ -9647,7 +9636,7 @@
         <v>0.11541</v>
       </c>
     </row>
-    <row r="210" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>492</v>
       </c>
@@ -9691,7 +9680,7 @@
         <v>0.11348999999999999</v>
       </c>
     </row>
-    <row r="211" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>491</v>
       </c>
@@ -9735,7 +9724,7 @@
         <v>0.11176</v>
       </c>
     </row>
-    <row r="212" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>490</v>
       </c>
@@ -9779,7 +9768,7 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="213" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>489</v>
       </c>
@@ -9823,7 +9812,7 @@
         <v>0.10833</v>
       </c>
     </row>
-    <row r="214" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>488</v>
       </c>
@@ -9867,7 +9856,7 @@
         <v>0.10682999999999999</v>
       </c>
     </row>
-    <row r="215" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>487</v>
       </c>
@@ -9911,7 +9900,7 @@
         <v>0.10519000000000001</v>
       </c>
     </row>
-    <row r="216" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>486</v>
       </c>
@@ -9955,7 +9944,7 @@
         <v>0.10367</v>
       </c>
     </row>
-    <row r="217" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>485</v>
       </c>
@@ -9999,7 +9988,7 @@
         <v>0.10185</v>
       </c>
     </row>
-    <row r="218" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>484</v>
       </c>
@@ -10043,7 +10032,7 @@
         <v>0.10008</v>
       </c>
     </row>
-    <row r="219" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>483</v>
       </c>
@@ -10087,7 +10076,7 @@
         <v>9.8659999999999998E-2</v>
       </c>
     </row>
-    <row r="220" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>482</v>
       </c>
@@ -10131,7 +10120,7 @@
         <v>9.7040000000000001E-2</v>
       </c>
     </row>
-    <row r="221" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>481</v>
       </c>
@@ -10175,7 +10164,7 @@
         <v>9.5380000000000006E-2</v>
       </c>
     </row>
-    <row r="222" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>480</v>
       </c>
@@ -10219,7 +10208,7 @@
         <v>9.3859999999999999E-2</v>
       </c>
     </row>
-    <row r="223" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>479</v>
       </c>
@@ -10263,7 +10252,7 @@
         <v>9.2119999999999994E-2</v>
       </c>
     </row>
-    <row r="224" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>478</v>
       </c>
@@ -10307,7 +10296,7 @@
         <v>9.0620000000000006E-2</v>
       </c>
     </row>
-    <row r="225" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>477</v>
       </c>
@@ -10351,7 +10340,7 @@
         <v>8.8770000000000002E-2</v>
       </c>
     </row>
-    <row r="226" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>476</v>
       </c>
@@ -10395,7 +10384,7 @@
         <v>8.7090000000000001E-2</v>
       </c>
     </row>
-    <row r="227" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>475</v>
       </c>
@@ -10439,7 +10428,7 @@
         <v>8.5720000000000005E-2</v>
       </c>
     </row>
-    <row r="228" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>474</v>
       </c>
@@ -10483,7 +10472,7 @@
         <v>8.4349999999999994E-2</v>
       </c>
     </row>
-    <row r="229" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>473</v>
       </c>
@@ -10527,7 +10516,7 @@
         <v>8.2610000000000003E-2</v>
       </c>
     </row>
-    <row r="230" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>472</v>
       </c>
@@ -10571,7 +10560,7 @@
         <v>8.1059999999999993E-2</v>
       </c>
     </row>
-    <row r="231" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>471</v>
       </c>
@@ -10615,7 +10604,7 @@
         <v>7.9530000000000003E-2</v>
       </c>
     </row>
-    <row r="232" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>470</v>
       </c>
@@ -10659,7 +10648,7 @@
         <v>7.8009999999999996E-2</v>
       </c>
     </row>
-    <row r="233" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>469</v>
       </c>
@@ -10703,7 +10692,7 @@
         <v>7.6619999999999994E-2</v>
       </c>
     </row>
-    <row r="234" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>468</v>
       </c>
@@ -10747,7 +10736,7 @@
         <v>7.5120000000000006E-2</v>
       </c>
     </row>
-    <row r="235" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>467</v>
       </c>
@@ -10791,7 +10780,7 @@
         <v>7.3950000000000002E-2</v>
       </c>
     </row>
-    <row r="236" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>466</v>
       </c>
@@ -10835,7 +10824,7 @@
         <v>7.2720000000000007E-2</v>
       </c>
     </row>
-    <row r="237" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>465</v>
       </c>
@@ -10879,7 +10868,7 @@
         <v>7.109E-2</v>
       </c>
     </row>
-    <row r="238" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>464</v>
       </c>
@@ -10923,7 +10912,7 @@
         <v>7.0099999999999996E-2</v>
       </c>
     </row>
-    <row r="239" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>463</v>
       </c>
@@ -10967,7 +10956,7 @@
         <v>6.905E-2</v>
       </c>
     </row>
-    <row r="240" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>462</v>
       </c>
@@ -11011,7 +11000,7 @@
         <v>6.8019999999999997E-2</v>
       </c>
     </row>
-    <row r="241" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>461</v>
       </c>
@@ -11055,7 +11044,7 @@
         <v>6.7339999999999997E-2</v>
       </c>
     </row>
-    <row r="242" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>460</v>
       </c>
@@ -11099,7 +11088,7 @@
         <v>6.6489999999999994E-2</v>
       </c>
     </row>
-    <row r="243" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>459</v>
       </c>
@@ -11143,7 +11132,7 @@
         <v>6.6049999999999998E-2</v>
       </c>
     </row>
-    <row r="244" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>458</v>
       </c>
@@ -11187,7 +11176,7 @@
         <v>6.5250000000000002E-2</v>
       </c>
     </row>
-    <row r="245" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>457</v>
       </c>
@@ -11231,7 +11220,7 @@
         <v>6.4630000000000007E-2</v>
       </c>
     </row>
-    <row r="246" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>456</v>
       </c>
@@ -11275,7 +11264,7 @@
         <v>6.4740000000000006E-2</v>
       </c>
     </row>
-    <row r="247" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>455</v>
       </c>
@@ -11319,7 +11308,7 @@
         <v>6.4680000000000001E-2</v>
       </c>
     </row>
-    <row r="248" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>454</v>
       </c>
@@ -11363,7 +11352,7 @@
         <v>6.4570000000000002E-2</v>
       </c>
     </row>
-    <row r="249" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>453</v>
       </c>
@@ -11407,7 +11396,7 @@
         <v>6.4799999999999996E-2</v>
       </c>
     </row>
-    <row r="250" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>452</v>
       </c>
@@ -11451,7 +11440,7 @@
         <v>6.5089999999999995E-2</v>
       </c>
     </row>
-    <row r="251" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>451</v>
       </c>
@@ -11495,7 +11484,7 @@
         <v>6.5420000000000006E-2</v>
       </c>
     </row>
-    <row r="252" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>450</v>
       </c>
@@ -11539,7 +11528,7 @@
         <v>6.6250000000000003E-2</v>
       </c>
     </row>
-    <row r="253" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>449</v>
       </c>
@@ -11583,7 +11572,7 @@
         <v>6.7000000000000004E-2</v>
       </c>
     </row>
-    <row r="254" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>448</v>
       </c>
@@ -11627,7 +11616,7 @@
         <v>6.7780000000000007E-2</v>
       </c>
     </row>
-    <row r="255" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>447</v>
       </c>
@@ -11671,7 +11660,7 @@
         <v>6.9459999999999994E-2</v>
       </c>
     </row>
-    <row r="256" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>446</v>
       </c>
@@ -11715,7 +11704,7 @@
         <v>7.0699999999999999E-2</v>
       </c>
     </row>
-    <row r="257" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>445</v>
       </c>
@@ -11759,7 +11748,7 @@
         <v>7.1739999999999998E-2</v>
       </c>
     </row>
-    <row r="258" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>444</v>
       </c>
@@ -11803,7 +11792,7 @@
         <v>7.3779999999999998E-2</v>
       </c>
     </row>
-    <row r="259" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>443</v>
       </c>
@@ -11847,7 +11836,7 @@
         <v>7.5569999999999998E-2</v>
       </c>
     </row>
-    <row r="260" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>442</v>
       </c>
@@ -11891,7 +11880,7 @@
         <v>7.7109999999999998E-2</v>
       </c>
     </row>
-    <row r="261" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>441</v>
       </c>
@@ -11935,7 +11924,7 @@
         <v>7.9670000000000005E-2</v>
       </c>
     </row>
-    <row r="262" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>440</v>
       </c>
@@ -11979,7 +11968,7 @@
         <v>8.2199999999999995E-2</v>
       </c>
     </row>
-    <row r="263" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>439</v>
       </c>
@@ -12023,7 +12012,7 @@
         <v>8.4449999999999997E-2</v>
       </c>
     </row>
-    <row r="264" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>438</v>
       </c>
@@ -12067,7 +12056,7 @@
         <v>8.727E-2</v>
       </c>
     </row>
-    <row r="265" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>437</v>
       </c>
@@ -12111,7 +12100,7 @@
         <v>8.9950000000000002E-2</v>
       </c>
     </row>
-    <row r="266" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>436</v>
       </c>
@@ -12155,7 +12144,7 @@
         <v>9.2380000000000004E-2</v>
       </c>
     </row>
-    <row r="267" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>435</v>
       </c>
@@ -12199,7 +12188,7 @@
         <v>9.5899999999999999E-2</v>
       </c>
     </row>
-    <row r="268" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>434</v>
       </c>
@@ -12243,7 +12232,7 @@
         <v>9.8530000000000006E-2</v>
       </c>
     </row>
-    <row r="269" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>433</v>
       </c>
@@ -12287,7 +12276,7 @@
         <v>0.1016</v>
       </c>
     </row>
-    <row r="270" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>432</v>
       </c>
@@ -12331,7 +12320,7 @@
         <v>0.10456</v>
       </c>
     </row>
-    <row r="271" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>431</v>
       </c>
@@ -12375,7 +12364,7 @@
         <v>0.10761</v>
       </c>
     </row>
-    <row r="272" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>430</v>
       </c>
@@ -12419,7 +12408,7 @@
         <v>0.11114</v>
       </c>
     </row>
-    <row r="273" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>429</v>
       </c>
@@ -12463,7 +12452,7 @@
         <v>0.11397</v>
       </c>
     </row>
-    <row r="274" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>428</v>
       </c>
@@ -12507,7 +12496,7 @@
         <v>0.11681</v>
       </c>
     </row>
-    <row r="275" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>427</v>
       </c>
@@ -12551,7 +12540,7 @@
         <v>0.11992</v>
       </c>
     </row>
-    <row r="276" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>426</v>
       </c>
@@ -12595,7 +12584,7 @@
         <v>0.12305000000000001</v>
       </c>
     </row>
-    <row r="277" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>425</v>
       </c>
@@ -12639,7 +12628,7 @@
         <v>0.12631000000000001</v>
       </c>
     </row>
-    <row r="278" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>424</v>
       </c>
@@ -12683,7 +12672,7 @@
         <v>0.12875</v>
       </c>
     </row>
-    <row r="279" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>423</v>
       </c>
@@ -12727,7 +12716,7 @@
         <v>0.13184999999999999</v>
       </c>
     </row>
-    <row r="280" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>422</v>
       </c>
@@ -12771,7 +12760,7 @@
         <v>0.13475000000000001</v>
       </c>
     </row>
-    <row r="281" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>421</v>
       </c>
@@ -12815,7 +12804,7 @@
         <v>0.13755999999999999</v>
       </c>
     </row>
-    <row r="282" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>420</v>
       </c>
@@ -12859,7 +12848,7 @@
         <v>0.14072000000000001</v>
       </c>
     </row>
-    <row r="283" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>419</v>
       </c>
@@ -12903,7 +12892,7 @@
         <v>0.14327999999999999</v>
       </c>
     </row>
-    <row r="284" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>418</v>
       </c>
@@ -12947,7 +12936,7 @@
         <v>0.14574999999999999</v>
       </c>
     </row>
-    <row r="285" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>417</v>
       </c>
@@ -12991,7 +12980,7 @@
         <v>0.14868000000000001</v>
       </c>
     </row>
-    <row r="286" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>416</v>
       </c>
@@ -13035,7 +13024,7 @@
         <v>0.15160999999999999</v>
       </c>
     </row>
-    <row r="287" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>415</v>
       </c>
@@ -13079,7 +13068,7 @@
         <v>0.15459000000000001</v>
       </c>
     </row>
-    <row r="288" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>414</v>
       </c>
@@ -13123,7 +13112,7 @@
         <v>0.15731000000000001</v>
       </c>
     </row>
-    <row r="289" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>413</v>
       </c>
@@ -13167,7 +13156,7 @@
         <v>0.16036</v>
       </c>
     </row>
-    <row r="290" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>412</v>
       </c>
@@ -13211,7 +13200,7 @@
         <v>0.16345000000000001</v>
       </c>
     </row>
-    <row r="291" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>411</v>
       </c>
@@ -13255,7 +13244,7 @@
         <v>0.16696</v>
       </c>
     </row>
-    <row r="292" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>410</v>
       </c>
@@ -13299,7 +13288,7 @@
         <v>0.17002999999999999</v>
       </c>
     </row>
-    <row r="293" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>409</v>
       </c>
@@ -13343,7 +13332,7 @@
         <v>0.17363999999999999</v>
       </c>
     </row>
-    <row r="294" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>408</v>
       </c>
@@ -13387,7 +13376,7 @@
         <v>0.17696999999999999</v>
       </c>
     </row>
-    <row r="295" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>407</v>
       </c>
@@ -13431,7 +13420,7 @@
         <v>0.18040999999999999</v>
       </c>
     </row>
-    <row r="296" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>406</v>
       </c>
@@ -13475,7 +13464,7 @@
         <v>0.18385000000000001</v>
       </c>
     </row>
-    <row r="297" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>405</v>
       </c>
@@ -13519,7 +13508,7 @@
         <v>0.18745000000000001</v>
       </c>
     </row>
-    <row r="298" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>404</v>
       </c>
@@ -13563,7 +13552,7 @@
         <v>0.19095000000000001</v>
       </c>
     </row>
-    <row r="299" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>403</v>
       </c>
@@ -13607,7 +13596,7 @@
         <v>0.19420999999999999</v>
       </c>
     </row>
-    <row r="300" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>402</v>
       </c>
@@ -13651,7 +13640,7 @@
         <v>0.19783999999999999</v>
       </c>
     </row>
-    <row r="301" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>401</v>
       </c>
@@ -13695,7 +13684,7 @@
         <v>0.20086000000000001</v>
       </c>
     </row>
-    <row r="302" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>400</v>
       </c>
@@ -13739,7 +13728,7 @@
         <v>0.20419999999999999</v>
       </c>
     </row>
-    <row r="303" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>399</v>
       </c>
@@ -13783,7 +13772,7 @@
         <v>0.20707</v>
       </c>
     </row>
-    <row r="304" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>398</v>
       </c>
@@ -13827,7 +13816,7 @@
         <v>0.21007999999999999</v>
       </c>
     </row>
-    <row r="305" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>397</v>
       </c>
@@ -13871,7 +13860,7 @@
         <v>0.21321000000000001</v>
       </c>
     </row>
-    <row r="306" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>396</v>
       </c>
@@ -13915,7 +13904,7 @@
         <v>0.21561</v>
       </c>
     </row>
-    <row r="307" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>395</v>
       </c>
@@ -13959,7 +13948,7 @@
         <v>0.21808</v>
       </c>
     </row>
-    <row r="308" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>394</v>
       </c>
@@ -14003,7 +13992,7 @@
         <v>0.22023999999999999</v>
       </c>
     </row>
-    <row r="309" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>393</v>
       </c>
@@ -14047,7 +14036,7 @@
         <v>0.22239</v>
       </c>
     </row>
-    <row r="310" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>392</v>
       </c>
@@ -14091,7 +14080,7 @@
         <v>0.22425999999999999</v>
       </c>
     </row>
-    <row r="311" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>391</v>
       </c>
@@ -14135,7 +14124,7 @@
         <v>0.22639000000000001</v>
       </c>
     </row>
-    <row r="312" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>390</v>
       </c>
@@ -14179,7 +14168,7 @@
         <v>0.22792999999999999</v>
       </c>
     </row>
-    <row r="313" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>389</v>
       </c>
@@ -14223,7 +14212,7 @@
         <v>0.22911999999999999</v>
       </c>
     </row>
-    <row r="314" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="314" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>388</v>
       </c>
@@ -14267,7 +14256,7 @@
         <v>0.23083999999999999</v>
       </c>
     </row>
-    <row r="315" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>387</v>
       </c>
@@ -14311,7 +14300,7 @@
         <v>0.23191999999999999</v>
       </c>
     </row>
-    <row r="316" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>386</v>
       </c>
@@ -14355,7 +14344,7 @@
         <v>0.23311000000000001</v>
       </c>
     </row>
-    <row r="317" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>385</v>
       </c>
@@ -14399,7 +14388,7 @@
         <v>0.23394000000000001</v>
       </c>
     </row>
-    <row r="318" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>384</v>
       </c>
@@ -14443,7 +14432,7 @@
         <v>0.23491999999999999</v>
       </c>
     </row>
-    <row r="319" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="319" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>383</v>
       </c>
@@ -14487,7 +14476,7 @@
         <v>0.2361</v>
       </c>
     </row>
-    <row r="320" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>382</v>
       </c>
@@ -14531,7 +14520,7 @@
         <v>0.23730999999999999</v>
       </c>
     </row>
-    <row r="321" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>381</v>
       </c>
@@ -14575,7 +14564,7 @@
         <v>0.23810999999999999</v>
       </c>
     </row>
-    <row r="322" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>380</v>
       </c>
@@ -14619,7 +14608,7 @@
         <v>0.23946000000000001</v>
       </c>
     </row>
-    <row r="323" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>379</v>
       </c>
@@ -14663,7 +14652,7 @@
         <v>0.24071999999999999</v>
       </c>
     </row>
-    <row r="324" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>378</v>
       </c>
@@ -14707,7 +14696,7 @@
         <v>0.24182999999999999</v>
       </c>
     </row>
-    <row r="325" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="325" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>377</v>
       </c>
@@ -14751,7 +14740,7 @@
         <v>0.24318999999999999</v>
       </c>
     </row>
-    <row r="326" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>376</v>
       </c>
@@ -14795,7 +14784,7 @@
         <v>0.24492</v>
       </c>
     </row>
-    <row r="327" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>375</v>
       </c>
@@ -14839,7 +14828,7 @@
         <v>0.24621999999999999</v>
       </c>
     </row>
-    <row r="328" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>374</v>
       </c>
@@ -14883,7 +14872,7 @@
         <v>0.24801000000000001</v>
       </c>
     </row>
-    <row r="329" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>373</v>
       </c>
@@ -14927,7 +14916,7 @@
         <v>0.25045000000000001</v>
       </c>
     </row>
-    <row r="330" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>372</v>
       </c>
@@ -14971,7 +14960,7 @@
         <v>0.25189</v>
       </c>
     </row>
-    <row r="331" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>371</v>
       </c>
@@ -15015,7 +15004,7 @@
         <v>0.25408999999999998</v>
       </c>
     </row>
-    <row r="332" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>370</v>
       </c>
@@ -15059,7 +15048,7 @@
         <v>0.25714999999999999</v>
       </c>
     </row>
-    <row r="333" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>369</v>
       </c>
@@ -15103,7 +15092,7 @@
         <v>0.25933</v>
       </c>
     </row>
-    <row r="334" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>368</v>
       </c>
@@ -15147,7 +15136,7 @@
         <v>0.26191999999999999</v>
       </c>
     </row>
-    <row r="335" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>367</v>
       </c>
@@ -15191,7 +15180,7 @@
         <v>0.26389000000000001</v>
       </c>
     </row>
-    <row r="336" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>366</v>
       </c>
@@ -15235,7 +15224,7 @@
         <v>0.2666</v>
       </c>
     </row>
-    <row r="337" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>365</v>
       </c>
@@ -15279,7 +15268,7 @@
         <v>0.26940999999999998</v>
       </c>
     </row>
-    <row r="338" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>364</v>
       </c>
@@ -15323,7 +15312,7 @@
         <v>0.27177000000000001</v>
       </c>
     </row>
-    <row r="339" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>363</v>
       </c>
@@ -15367,7 +15356,7 @@
         <v>0.27448</v>
       </c>
     </row>
-    <row r="340" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>362</v>
       </c>
@@ -15411,7 +15400,7 @@
         <v>0.27711999999999998</v>
       </c>
     </row>
-    <row r="341" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>361</v>
       </c>
@@ -15455,7 +15444,7 @@
         <v>0.28032000000000001</v>
       </c>
     </row>
-    <row r="342" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A342">
         <v>360</v>
       </c>
@@ -15499,7 +15488,7 @@
         <v>0.28339999999999999</v>
       </c>
     </row>
-    <row r="343" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>359</v>
       </c>
@@ -15543,7 +15532,7 @@
         <v>0.28664000000000001</v>
       </c>
     </row>
-    <row r="344" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A344">
         <v>358</v>
       </c>
@@ -15587,7 +15576,7 @@
         <v>0.29025000000000001</v>
       </c>
     </row>
-    <row r="345" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="345" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A345">
         <v>357</v>
       </c>
@@ -15631,7 +15620,7 @@
         <v>0.29393999999999998</v>
       </c>
     </row>
-    <row r="346" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A346">
         <v>356</v>
       </c>
@@ -15675,7 +15664,7 @@
         <v>0.29846</v>
       </c>
     </row>
-    <row r="347" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A347">
         <v>355</v>
       </c>
@@ -15719,7 +15708,7 @@
         <v>0.30370000000000003</v>
       </c>
     </row>
-    <row r="348" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A348">
         <v>354</v>
       </c>
@@ -15763,7 +15752,7 @@
         <v>0.30925999999999998</v>
       </c>
     </row>
-    <row r="349" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>353</v>
       </c>
@@ -15807,7 +15796,7 @@
         <v>0.31525999999999998</v>
       </c>
     </row>
-    <row r="350" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A350">
         <v>352</v>
       </c>
@@ -15851,7 +15840,7 @@
         <v>0.32199</v>
       </c>
     </row>
-    <row r="351" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>351</v>
       </c>
@@ -15895,7 +15884,7 @@
         <v>0.33008999999999999</v>
       </c>
     </row>
-    <row r="352" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A352">
         <v>350</v>
       </c>
@@ -15939,7 +15928,7 @@
         <v>0.33738000000000001</v>
       </c>
     </row>
-    <row r="353" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="353" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C353">
         <v>399</v>
       </c>
@@ -15977,7 +15966,7 @@
         <v>0.34609000000000001</v>
       </c>
     </row>
-    <row r="354" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="354" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C354">
         <v>398</v>
       </c>
@@ -16015,7 +16004,7 @@
         <v>0.35424</v>
       </c>
     </row>
-    <row r="355" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="355" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C355">
         <v>397</v>
       </c>
@@ -16053,7 +16042,7 @@
         <v>0.36220999999999998</v>
       </c>
     </row>
-    <row r="356" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="356" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C356">
         <v>396</v>
       </c>
@@ -16091,7 +16080,7 @@
         <v>0.36963000000000001</v>
       </c>
     </row>
-    <row r="357" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="357" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C357">
         <v>395</v>
       </c>
@@ -16129,7 +16118,7 @@
         <v>0.37702000000000002</v>
       </c>
     </row>
-    <row r="358" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="358" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C358">
         <v>394</v>
       </c>
@@ -16167,7 +16156,7 @@
         <v>0.38366</v>
       </c>
     </row>
-    <row r="359" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="359" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C359">
         <v>393</v>
       </c>
@@ -16205,7 +16194,7 @@
         <v>0.38840000000000002</v>
       </c>
     </row>
-    <row r="360" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="360" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C360">
         <v>392</v>
       </c>
@@ -16243,7 +16232,7 @@
         <v>0.39311000000000001</v>
       </c>
     </row>
-    <row r="361" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="361" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C361">
         <v>391</v>
       </c>
@@ -16281,7 +16270,7 @@
         <v>0.39651999999999998</v>
       </c>
     </row>
-    <row r="362" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="362" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C362">
         <v>390</v>
       </c>
@@ -16319,7 +16308,7 @@
         <v>0.39883000000000002</v>
       </c>
     </row>
-    <row r="363" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="363" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C363">
         <v>389</v>
       </c>
@@ -16357,7 +16346,7 @@
         <v>0.39995999999999998</v>
       </c>
     </row>
-    <row r="364" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="364" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C364">
         <v>388</v>
       </c>
@@ -16395,7 +16384,7 @@
         <v>0.39996999999999999</v>
       </c>
     </row>
-    <row r="365" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="365" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C365">
         <v>387</v>
       </c>
@@ -16433,7 +16422,7 @@
         <v>0.39962999999999999</v>
       </c>
     </row>
-    <row r="366" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="366" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C366">
         <v>386</v>
       </c>
@@ -16471,7 +16460,7 @@
         <v>0.39813999999999999</v>
       </c>
     </row>
-    <row r="367" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="367" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C367">
         <v>385</v>
       </c>
@@ -16509,7 +16498,7 @@
         <v>0.39665</v>
       </c>
     </row>
-    <row r="368" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="368" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C368">
         <v>384</v>
       </c>
@@ -16547,7 +16536,7 @@
         <v>0.39466000000000001</v>
       </c>
     </row>
-    <row r="369" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="369" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C369">
         <v>383</v>
       </c>
@@ -16585,7 +16574,7 @@
         <v>0.39149</v>
       </c>
     </row>
-    <row r="370" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="370" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C370">
         <v>382</v>
       </c>
@@ -16623,7 +16612,7 @@
         <v>0.38941999999999999</v>
       </c>
     </row>
-    <row r="371" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="371" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C371">
         <v>381</v>
       </c>
@@ -16661,7 +16650,7 @@
         <v>0.38708999999999999</v>
       </c>
     </row>
-    <row r="372" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="372" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C372">
         <v>380</v>
       </c>
@@ -16699,7 +16688,7 @@
         <v>0.38434000000000001</v>
       </c>
     </row>
-    <row r="373" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="373" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C373">
         <v>379</v>
       </c>
@@ -16737,7 +16726,7 @@
         <v>0.38174999999999998</v>
       </c>
     </row>
-    <row r="374" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="374" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C374">
         <v>378</v>
       </c>
@@ -16775,7 +16764,7 @@
         <v>0.37948999999999999</v>
       </c>
     </row>
-    <row r="375" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="375" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C375">
         <v>377</v>
       </c>
@@ -16813,7 +16802,7 @@
         <v>0.37747000000000003</v>
       </c>
     </row>
-    <row r="376" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="376" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C376">
         <v>376</v>
       </c>
@@ -16851,7 +16840,7 @@
         <v>0.37614999999999998</v>
       </c>
     </row>
-    <row r="377" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="377" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C377">
         <v>375</v>
       </c>
@@ -16889,7 +16878,7 @@
         <v>0.37365999999999999</v>
       </c>
     </row>
-    <row r="378" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="378" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C378">
         <v>374</v>
       </c>
@@ -16927,7 +16916,7 @@
         <v>0.37128</v>
       </c>
     </row>
-    <row r="379" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="379" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C379">
         <v>373</v>
       </c>
@@ -16965,7 +16954,7 @@
         <v>0.37043999999999999</v>
       </c>
     </row>
-    <row r="380" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="380" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C380">
         <v>372</v>
       </c>
@@ -17003,7 +16992,7 @@
         <v>0.36923</v>
       </c>
     </row>
-    <row r="381" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="381" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C381">
         <v>371</v>
       </c>
@@ -17041,7 +17030,7 @@
         <v>0.36753999999999998</v>
       </c>
     </row>
-    <row r="382" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="382" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C382">
         <v>370</v>
       </c>
@@ -17079,7 +17068,7 @@
         <v>0.36592000000000002</v>
       </c>
     </row>
-    <row r="383" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="383" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C383">
         <v>369</v>
       </c>
@@ -17117,7 +17106,7 @@
         <v>0.36386000000000002</v>
       </c>
     </row>
-    <row r="384" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="384" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C384">
         <v>368</v>
       </c>
@@ -17155,7 +17144,7 @@
         <v>0.36109000000000002</v>
       </c>
     </row>
-    <row r="385" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="385" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C385">
         <v>367</v>
       </c>
@@ -17193,7 +17182,7 @@
         <v>0.35843000000000003</v>
       </c>
     </row>
-    <row r="386" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="386" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C386">
         <v>366</v>
       </c>
@@ -17231,7 +17220,7 @@
         <v>0.35474</v>
       </c>
     </row>
-    <row r="387" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="387" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C387">
         <v>365</v>
       </c>
@@ -17269,7 +17258,7 @@
         <v>0.35189999999999999</v>
       </c>
     </row>
-    <row r="388" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="388" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C388">
         <v>364</v>
       </c>
@@ -17307,7 +17296,7 @@
         <v>0.34761999999999998</v>
       </c>
     </row>
-    <row r="389" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="389" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C389">
         <v>363</v>
       </c>
@@ -17345,7 +17334,7 @@
         <v>0.34366000000000002</v>
       </c>
     </row>
-    <row r="390" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="390" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C390">
         <v>362</v>
       </c>
@@ -17383,7 +17372,7 @@
         <v>0.33865000000000001</v>
       </c>
     </row>
-    <row r="391" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="391" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C391">
         <v>361</v>
       </c>
@@ -17421,7 +17410,7 @@
         <v>0.33467999999999998</v>
       </c>
     </row>
-    <row r="392" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="392" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C392">
         <v>360</v>
       </c>
@@ -17459,7 +17448,7 @@
         <v>0.32911000000000001</v>
       </c>
     </row>
-    <row r="393" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="393" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C393">
         <v>359</v>
       </c>
@@ -17497,7 +17486,7 @@
         <v>0.32534999999999997</v>
       </c>
     </row>
-    <row r="394" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="394" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C394">
         <v>358</v>
       </c>
@@ -17535,7 +17524,7 @@
         <v>0.31961000000000001</v>
       </c>
     </row>
-    <row r="395" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="395" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C395">
         <v>357</v>
       </c>
@@ -17573,7 +17562,7 @@
         <v>0.31464999999999999</v>
       </c>
     </row>
-    <row r="396" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="396" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C396">
         <v>356</v>
       </c>
@@ -17611,7 +17600,7 @@
         <v>0.311</v>
       </c>
     </row>
-    <row r="397" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="397" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C397">
         <v>355</v>
       </c>
@@ -17649,7 +17638,7 @@
         <v>0.30553000000000002</v>
       </c>
     </row>
-    <row r="398" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="398" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C398">
         <v>354</v>
       </c>
@@ -17687,7 +17676,7 @@
         <v>0.30185000000000001</v>
       </c>
     </row>
-    <row r="399" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="399" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C399">
         <v>353</v>
       </c>
@@ -17725,7 +17714,7 @@
         <v>0.29873</v>
       </c>
     </row>
-    <row r="400" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="400" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C400">
         <v>352</v>
       </c>
@@ -17763,7 +17752,7 @@
         <v>0.29538999999999999</v>
       </c>
     </row>
-    <row r="401" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="401" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C401">
         <v>351</v>
       </c>
@@ -17801,7 +17790,7 @@
         <v>0.29257</v>
       </c>
     </row>
-    <row r="402" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="402" spans="3:17" x14ac:dyDescent="0.3">
       <c r="C402">
         <v>350</v>
       </c>
@@ -17839,7 +17828,7 @@
         <v>0.29091</v>
       </c>
     </row>
-    <row r="403" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="403" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J403">
         <v>399</v>
       </c>
@@ -17856,7 +17845,7 @@
         <v>1.3998200000000001</v>
       </c>
     </row>
-    <row r="404" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="404" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J404">
         <v>398</v>
       </c>
@@ -17873,7 +17862,7 @@
         <v>1.37934</v>
       </c>
     </row>
-    <row r="405" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="405" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J405">
         <v>397</v>
       </c>
@@ -17890,7 +17879,7 @@
         <v>1.37365</v>
       </c>
     </row>
-    <row r="406" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="406" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J406">
         <v>396</v>
       </c>
@@ -17907,7 +17896,7 @@
         <v>1.35945</v>
       </c>
     </row>
-    <row r="407" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="407" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J407">
         <v>395</v>
       </c>
@@ -17924,7 +17913,7 @@
         <v>1.34338</v>
       </c>
     </row>
-    <row r="408" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="408" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J408">
         <v>394</v>
       </c>
@@ -17941,7 +17930,7 @@
         <v>1.3441099999999999</v>
       </c>
     </row>
-    <row r="409" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="409" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J409">
         <v>393</v>
       </c>
@@ -17958,7 +17947,7 @@
         <v>1.3344</v>
       </c>
     </row>
-    <row r="410" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="410" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J410">
         <v>392</v>
       </c>
@@ -17975,7 +17964,7 @@
         <v>1.3264899999999999</v>
       </c>
     </row>
-    <row r="411" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="411" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J411">
         <v>391</v>
       </c>
@@ -17992,7 +17981,7 @@
         <v>1.3129599999999999</v>
       </c>
     </row>
-    <row r="412" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="412" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J412">
         <v>390</v>
       </c>
@@ -18009,7 +17998,7 @@
         <v>1.2990200000000001</v>
       </c>
     </row>
-    <row r="413" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="413" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J413">
         <v>389</v>
       </c>
@@ -18026,7 +18015,7 @@
         <v>1.29416</v>
       </c>
     </row>
-    <row r="414" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="414" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J414">
         <v>388</v>
       </c>
@@ -18043,7 +18032,7 @@
         <v>1.2913300000000001</v>
       </c>
     </row>
-    <row r="415" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="415" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J415">
         <v>387</v>
       </c>
@@ -18060,7 +18049,7 @@
         <v>1.2735300000000001</v>
       </c>
     </row>
-    <row r="416" spans="3:17" x14ac:dyDescent="0.2">
+    <row r="416" spans="3:17" x14ac:dyDescent="0.3">
       <c r="J416">
         <v>386</v>
       </c>
@@ -18077,7 +18066,7 @@
         <v>1.27024</v>
       </c>
     </row>
-    <row r="417" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="417" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J417">
         <v>385</v>
       </c>
@@ -18094,7 +18083,7 @@
         <v>1.2551000000000001</v>
       </c>
     </row>
-    <row r="418" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="418" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J418">
         <v>384</v>
       </c>
@@ -18111,7 +18100,7 @@
         <v>1.25556</v>
       </c>
     </row>
-    <row r="419" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="419" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J419">
         <v>383</v>
       </c>
@@ -18128,7 +18117,7 @@
         <v>1.24624</v>
       </c>
     </row>
-    <row r="420" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="420" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J420">
         <v>382</v>
       </c>
@@ -18145,7 +18134,7 @@
         <v>1.22898</v>
       </c>
     </row>
-    <row r="421" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="421" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J421">
         <v>381</v>
       </c>
@@ -18162,7 +18151,7 @@
         <v>1.2242500000000001</v>
       </c>
     </row>
-    <row r="422" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="422" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J422">
         <v>380</v>
       </c>
@@ -18179,7 +18168,7 @@
         <v>1.2234499999999999</v>
       </c>
     </row>
-    <row r="423" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="423" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J423">
         <v>379</v>
       </c>
@@ -18196,7 +18185,7 @@
         <v>1.2099299999999999</v>
       </c>
     </row>
-    <row r="424" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="424" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J424">
         <v>378</v>
       </c>
@@ -18213,7 +18202,7 @@
         <v>1.2067699999999999</v>
       </c>
     </row>
-    <row r="425" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="425" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J425">
         <v>377</v>
       </c>
@@ -18230,7 +18219,7 @@
         <v>1.1940200000000001</v>
       </c>
     </row>
-    <row r="426" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="426" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J426">
         <v>376</v>
       </c>
@@ -18247,7 +18236,7 @@
         <v>1.1779999999999999</v>
       </c>
     </row>
-    <row r="427" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="427" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J427">
         <v>375</v>
       </c>
@@ -18264,7 +18253,7 @@
         <v>1.1782600000000001</v>
       </c>
     </row>
-    <row r="428" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="428" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J428">
         <v>374</v>
       </c>
@@ -18281,7 +18270,7 @@
         <v>1.15866</v>
       </c>
     </row>
-    <row r="429" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="429" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J429">
         <v>373</v>
       </c>
@@ -18298,7 +18287,7 @@
         <v>1.1461699999999999</v>
       </c>
     </row>
-    <row r="430" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="430" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J430">
         <v>372</v>
       </c>
@@ -18315,7 +18304,7 @@
         <v>1.1336299999999999</v>
       </c>
     </row>
-    <row r="431" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="431" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J431">
         <v>371</v>
       </c>
@@ -18332,7 +18321,7 @@
         <v>1.14272</v>
       </c>
     </row>
-    <row r="432" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="432" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J432">
         <v>370</v>
       </c>
@@ -18349,7 +18338,7 @@
         <v>1.1237900000000001</v>
       </c>
     </row>
-    <row r="433" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="433" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J433">
         <v>369</v>
       </c>
@@ -18366,7 +18355,7 @@
         <v>1.1193900000000001</v>
       </c>
     </row>
-    <row r="434" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="434" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J434">
         <v>368</v>
       </c>
@@ -18383,7 +18372,7 @@
         <v>1.1147899999999999</v>
       </c>
     </row>
-    <row r="435" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="435" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J435">
         <v>367</v>
       </c>
@@ -18400,7 +18389,7 @@
         <v>1.1145700000000001</v>
       </c>
     </row>
-    <row r="436" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="436" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J436">
         <v>366</v>
       </c>
@@ -18417,7 +18406,7 @@
         <v>1.1006199999999999</v>
       </c>
     </row>
-    <row r="437" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="437" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J437">
         <v>365</v>
       </c>
@@ -18434,7 +18423,7 @@
         <v>1.0947499999999999</v>
       </c>
     </row>
-    <row r="438" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="438" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J438">
         <v>364</v>
       </c>
@@ -18451,7 +18440,7 @@
         <v>1.09646</v>
       </c>
     </row>
-    <row r="439" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="439" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J439">
         <v>363</v>
       </c>
@@ -18468,7 +18457,7 @@
         <v>1.1001799999999999</v>
       </c>
     </row>
-    <row r="440" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="440" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J440">
         <v>362</v>
       </c>
@@ -18485,7 +18474,7 @@
         <v>1.10097</v>
       </c>
     </row>
-    <row r="441" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="441" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J441">
         <v>361</v>
       </c>
@@ -18502,7 +18491,7 @@
         <v>1.08606</v>
       </c>
     </row>
-    <row r="442" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="442" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J442">
         <v>360</v>
       </c>
@@ -18519,7 +18508,7 @@
         <v>1.0843499999999999</v>
       </c>
     </row>
-    <row r="443" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="443" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J443">
         <v>359</v>
       </c>
@@ -18536,7 +18525,7 @@
         <v>1.0848100000000001</v>
       </c>
     </row>
-    <row r="444" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="444" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J444">
         <v>358</v>
       </c>
@@ -18553,7 +18542,7 @@
         <v>1.09419</v>
       </c>
     </row>
-    <row r="445" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="445" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J445">
         <v>357</v>
       </c>
@@ -18570,7 +18559,7 @@
         <v>1.08284</v>
       </c>
     </row>
-    <row r="446" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="446" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J446">
         <v>356</v>
       </c>
@@ -18587,7 +18576,7 @@
         <v>1.08867</v>
       </c>
     </row>
-    <row r="447" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="447" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J447">
         <v>355</v>
       </c>
@@ -18604,7 +18593,7 @@
         <v>1.0967800000000001</v>
       </c>
     </row>
-    <row r="448" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="448" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J448">
         <v>354</v>
       </c>
@@ -18621,7 +18610,7 @@
         <v>1.1008899999999999</v>
       </c>
     </row>
-    <row r="449" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="449" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J449">
         <v>353</v>
       </c>
@@ -18638,7 +18627,7 @@
         <v>1.09859</v>
       </c>
     </row>
-    <row r="450" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="450" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J450">
         <v>352</v>
       </c>
@@ -18655,7 +18644,7 @@
         <v>1.1096299999999999</v>
       </c>
     </row>
-    <row r="451" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="451" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J451">
         <v>351</v>
       </c>
@@ -18672,7 +18661,7 @@
         <v>1.1181300000000001</v>
       </c>
     </row>
-    <row r="452" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="452" spans="10:14" x14ac:dyDescent="0.3">
       <c r="J452">
         <v>350</v>
       </c>
@@ -18689,7 +18678,7 @@
         <v>1.1290500000000001</v>
       </c>
     </row>
-    <row r="453" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="453" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K453" t="s">
         <v>6</v>
       </c>
@@ -18703,7 +18692,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="454" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="454" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K454" t="s">
         <v>6</v>
       </c>
@@ -18717,7 +18706,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="455" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="455" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K455" t="s">
         <v>6</v>
       </c>
@@ -18731,7 +18720,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="456" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="456" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K456" t="s">
         <v>6</v>
       </c>
@@ -18745,7 +18734,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="457" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="457" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K457" t="s">
         <v>6</v>
       </c>
@@ -18759,7 +18748,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="458" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="458" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K458" t="s">
         <v>6</v>
       </c>
@@ -18773,7 +18762,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="459" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="459" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K459" t="s">
         <v>6</v>
       </c>
@@ -18787,7 +18776,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="460" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="460" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K460" t="s">
         <v>6</v>
       </c>
@@ -18801,7 +18790,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="461" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="461" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K461" t="s">
         <v>6</v>
       </c>
@@ -18815,7 +18804,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="462" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="462" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K462" t="s">
         <v>6</v>
       </c>
@@ -18829,7 +18818,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="463" spans="10:14" x14ac:dyDescent="0.2">
+    <row r="463" spans="10:14" x14ac:dyDescent="0.3">
       <c r="K463" t="s">
         <v>6</v>
       </c>
@@ -18851,210 +18840,210 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4614EA90-BDDA-EF4C-BBB4-04C3B376725D}">
   <dimension ref="B2:B70"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B61" s="1"/>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B70" s="1"/>
     </row>
   </sheetData>

</xml_diff>